<commit_message>
fix common set cell excel and fix format excel inventory, change name of quantity report
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportInventoryProductTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportInventoryProductTemplate.xlsx
@@ -467,7 +467,13 @@
   <dimension ref="A1:R1"/>
   <sheetFormatPr defaultColWidth="22" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="22" style="1"/>
+    <col min="1" max="1" width="22" style="1"/>
+    <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="22" style="1"/>
+    <col min="5" max="5" width="34" style="1" customWidth="1"/>
+    <col min="6" max="6" width="33.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.5703125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="22" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>